<commit_message>
still battling with the ministry of health
</commit_message>
<xml_diff>
--- a/Budget/data/budget_2022.xlsx
+++ b/Budget/data/budget_2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\NLP\anambra\Budget\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59A7BFE7-07CA-4A96-B7BD-A689F4709338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDDB7CA-F5CD-4F5A-BD83-BB4246DDA57A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9AA9ED6E-368D-482D-9C64-CEA0551C5F34}"/>
   </bookViews>
@@ -519,8 +519,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F514F26-19E1-4C5D-B90E-ADD6D49F7504}">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>